<commit_message>
tidying up code 3
</commit_message>
<xml_diff>
--- a/output/cost_estimates.xlsx
+++ b/output/cost_estimates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lh667\PersonalGitHub\MINA_TB\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A1F39FA-BC3D-459E-A783-56488D5998FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43304ED-AB36-4FA8-8BC0-0D80BF32BD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F819D8E4-99FC-45BB-9B6D-6F77878519FC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F819D8E4-99FC-45BB-9B6D-6F77878519FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -321,15 +321,39 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -337,30 +361,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -709,42 +709,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="9" t="s">
+      <c r="D1" s="4"/>
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="10"/>
+      <c r="F1" s="4"/>
     </row>
     <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="13" t="s">
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="9" t="s">
         <v>11</v>
       </c>
       <c r="G3" t="s">
@@ -770,32 +770,24 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="16"/>
+      <c r="A4" s="16"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="10"/>
     </row>
     <row r="5" spans="1:13" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="11" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="2">
-        <v>61452</v>
-      </c>
-      <c r="D5" s="2">
-        <v>46875</v>
-      </c>
-      <c r="E5" s="2">
-        <v>682</v>
-      </c>
-      <c r="F5" s="2">
-        <v>18554</v>
-      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
       <c r="I5">
         <f>G5-H5</f>
         <v>0</v>
@@ -810,22 +802,14 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="5"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
-        <v>52147</v>
-      </c>
-      <c r="D6" s="2">
-        <v>40941</v>
-      </c>
-      <c r="E6" s="2">
-        <v>717</v>
-      </c>
-      <c r="F6" s="2">
-        <v>21670</v>
-      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
       <c r="I6">
         <f t="shared" ref="I6:I10" si="2">G6-H6</f>
         <v>0</v>
@@ -840,22 +824,14 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="4"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="2">
-        <v>49527</v>
-      </c>
-      <c r="D7" s="2">
-        <v>37440</v>
-      </c>
-      <c r="E7" s="2">
-        <v>691</v>
-      </c>
-      <c r="F7" s="2">
-        <v>23654</v>
-      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
       <c r="I7">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -870,24 +846,16 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="2">
-        <v>91588</v>
-      </c>
-      <c r="D8" s="2">
-        <v>71988</v>
-      </c>
-      <c r="E8" s="2">
-        <v>666</v>
-      </c>
-      <c r="F8" s="2">
-        <v>16731</v>
-      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
       <c r="I8">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -902,22 +870,14 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="5"/>
+      <c r="A9" s="12"/>
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="2">
-        <v>61844</v>
-      </c>
-      <c r="D9" s="2">
-        <v>49434</v>
-      </c>
-      <c r="E9" s="2">
-        <v>674</v>
-      </c>
-      <c r="F9" s="2">
-        <v>20540</v>
-      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
       <c r="I9">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -932,22 +892,14 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="4"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="2">
-        <v>55415</v>
-      </c>
-      <c r="D10" s="2">
-        <v>41759</v>
-      </c>
-      <c r="E10" s="2">
-        <v>718</v>
-      </c>
-      <c r="F10" s="2">
-        <v>23050</v>
-      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
       <c r="I10">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -963,16 +915,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A1:A4"/>
+    <mergeCell ref="B1:B4"/>
+    <mergeCell ref="C1:D2"/>
     <mergeCell ref="E1:F2"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A1:A4"/>
-    <mergeCell ref="B1:B4"/>
-    <mergeCell ref="C1:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>